<commit_message>
E-book Excel : captures agrandies pour téléphone, repères recalés, intro compactée
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T8L22svZaEaGYSwza4q3Yc
</commit_message>
<xml_diff>
--- a/produits/preuves/sortie/nb-si-casse/nb-si-casse.xlsx
+++ b/produits/preuves/sortie/nb-si-casse/nb-si-casse.xlsx
@@ -273,10 +273,11 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8.97"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="4.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.97"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="7.76"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>